<commit_message>
Technical Change : Changed sharepoint download argument
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UiPath\S4_Hana\Non-BSO\AT_DRS_process\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0101734D-2154-4414-A6F2-A37FF5BAF25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F48ACCDD-C73C-41A7-A8AE-65E6932FFFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -235,9 +235,6 @@
     <t>SP_SKU_RelativeURL</t>
   </si>
   <si>
-    <t>Shared%20Documents/General/</t>
-  </si>
-  <si>
     <t>https://cchellenic.sharepoint.com/sites/SKUDashboardAT/</t>
   </si>
   <si>
@@ -296,6 +293,9 @@
   </si>
   <si>
     <t>RPAPRD1_SharePoint</t>
+  </si>
+  <si>
+    <t>https://cchellenic.sharepoint.com/sites/SKUDashboardAT/Shared%20Documents/General/</t>
   </si>
 </sst>
 </file>
@@ -360,9 +360,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,12 +676,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z997"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="62.85546875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.5703125" customWidth="1"/>
+    <col min="1" max="1" width="43.5546875" customWidth="1"/>
+    <col min="2" max="2" width="62.88671875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="81.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -731,7 +729,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
@@ -741,7 +739,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="30">
+    <row r="5" spans="1:26" ht="28.8">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -822,7 +820,7 @@
         <v>56</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
@@ -830,7 +828,7 @@
         <v>58</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
@@ -854,87 +852,87 @@
         <v>63</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>67</v>
+      <c r="B21" s="8" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>66</v>
+      <c r="B22" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
       <c r="A27" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
@@ -1918,12 +1916,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.5703125" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1960,7 +1958,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1971,7 +1969,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -2085,7 +2083,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="28.8">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -3079,12 +3077,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.7109375" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" customWidth="1"/>
-    <col min="3" max="3" width="60.42578125" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" customWidth="1"/>
+    <col min="3" max="3" width="60.44140625" customWidth="1"/>
+    <col min="4" max="26" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">

</xml_diff>